<commit_message>
text and format edits 4/26
</commit_message>
<xml_diff>
--- a/Concert Data.xlsx
+++ b/Concert Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mariacatoni/Documents/GitHub/final-project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FF1B779E-3EA9-364C-9EE3-60AAA25B8D81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63A2AFE3-1EAF-704E-A5C1-EC0B82DD5953}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5000" yWindow="780" windowWidth="29200" windowHeight="20280" xr2:uid="{C02E234E-A0E1-2146-80AB-BB1A5A023047}"/>
+    <workbookView xWindow="9600" yWindow="780" windowWidth="24600" windowHeight="20320" xr2:uid="{C02E234E-A0E1-2146-80AB-BB1A5A023047}"/>
   </bookViews>
   <sheets>
     <sheet name="Concerts by artist" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="951" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1037" uniqueCount="239">
   <si>
     <t>Date</t>
   </si>
@@ -534,6 +534,228 @@
   </si>
   <si>
     <t>Ela Minus</t>
+  </si>
+  <si>
+    <t>Setlist</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/ionnalee/2025/elsewhere-brooklyn-ny-6b588aea.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/lady-gaga/2025/madison-square-garden-new-york-ny-1b587550.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/blackpink/2025/citi-field-queens-ny-1b5b9544.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/charli-xcx/2025/barclays-center-brooklyn-ny-b5e75ea.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/dir-en-grey/2025/the-belasco-los-angeles-ca-6b508686.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/dir-en-grey/2025/the-belasco-los-angeles-ca-6b508682.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/xg/2024/madison-square-garden-the-theater-at-madison-square-garden-new-york-ny-735672ed.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/idle/2024/ubs-arena-elmont-ny-63578243.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/kard/2023/madison-square-garden-the-theater-at-madison-square-garden-new-york-ny-43a4bfff.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/caroline-polachek/2023/radio-city-music-hall-new-york-ny-43b93f63.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/epik-high/2023/hammerstein-ballroom-new-york-ny-3bbb52b.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/the-last-rockstars/2023/hammerstein-ballroom-new-york-ny-4bbd17de.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/lady-gaga/2022/metlife-stadium-east-rutherford-nj-3b39167.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/charli-xcx/2022/hammerstein-ballroom-new-york-ny-23b61013.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/charli-xcx/2022/hammerstein-ballroom-new-york-ny-33b61885.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/charli-xcx/2021/le-poisson-rouge-new-york-ny-538df3a1.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/dir-en-grey/2019/the-gramercy-theatre-new-york-ny-739bbea9.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/fka-twigs/2019/kings-theatre-brooklyn-ny-239af0b7.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/lady-gaga/2019/park-theater-at-park-mgm-las-vegas-nv-6b9dfaea.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/lady-gaga/2019/park-theater-at-park-mgm-las-vegas-nv-b9dfdfa.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/marina/2019/central-park-summerstage-new-york-ny-639cf28b.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/charli-xcx/2019/the-rooftop-at-pier-17-new-york-ny-73916aa5.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/bjork/2019/the-shed-new-york-ny-2390304b.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/fka-twigs/2019/park-avenue-armory-new-york-ny-23902893.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/allie-x/2019/bowery-ballroom-new-york-ny-6b935aea.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/ionnalee/2019/bowery-ballroom-new-york-ny-6b93567a.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/ionnalee/2018/music-hall-of-williamsburg-brooklyn-ny-33e80cf1.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/lorde/2018/barclays-center-brooklyn-ny-13ecbdcd.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/lady-gaga/2017/capital-one-arena-washington-dc-43e0eb2f.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/lady-gaga/2017/citi-field-queens-ny-53e293bd.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/lady-gaga/2017/citi-field-queens-ny-2be294aa.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/gdragon/2017/barclays-center-brooklyn-ny-7be5e210.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/perfume/2016/hammerstein-ballroom-new-york-ny-5bfc77bc.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/girls-generation/2015/prudential-center-newark-nj-23f24813.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/vixx/2015/prudential-center-newark-nj-53bb635d.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/teen-top/2015/prudential-center-newark-nj-43bb6353.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/aoa/2015/prudential-center-newark-nj-13ab590d.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/vamps/2015/best-buy-theater-new-york-ny-6bc80a96.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/perfume/2014/hammerstein-ballroom-new-york-ny-7bcd12ac.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/yelle/2014/irving-plaza-new-york-ny-63cc9e07.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/royksopp-and-robyn/2014/pier-97-hudson-river-park-new-york-ny-23ce145f.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/girls-generation/2014/los-angeles-sports-arena-los-angeles-ca-4bcef3aa.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/bts/2014/los-angeles-sports-arena-los-angeles-ca-3bf1c404.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/cnblue/2014/los-angeles-sports-arena-los-angeles-ca-4baaff06.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/spica/2014/los-angeles-sports-arena-los-angeles-ca-43aafffb.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/gdragon/2014/los-angeles-sports-arena-los-angeles-ca-13b2c509.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/iu/2014/los-angeles-sports-arena-los-angeles-ca-5baaff14.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/vixx/2014/los-angeles-sports-arena-los-angeles-ca-53aaff0d.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/b1a4/2014/los-angeles-sports-arena-los-angeles-ca-5baaff0c.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/teen-top/2014/los-angeles-sports-arena-los-angeles-ca-4baaff02.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/lorde/2014/roseland-ballroom-new-york-ny-3c2e14b.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/infinite/2013/hammerstein-ballroom-new-york-ny-7b9662d0.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/2ne1/2012/prudential-center-newark-nj-33dc1c15.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/the-cranberries/2012/terminal-5-new-york-ny-13de4189.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/larc-en-ciel/2012/madison-square-garden-new-york-ny-4bde2f2e.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/dir-en-grey/2011/irving-plaza-new-york-ny-1bd119a0.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/dir-en-grey/2011/sonar-baltimore-md-43d123e7.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/smtown/2010/staples-center-los-angeles-ca-1b5625fc.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/beirut/2011/terminal-5-new-york-ny-6bd01aca.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/girugamesh/2011/crash-mansion-new-york-ny-4bd3432e.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/royksopp/2011/music-hall-of-williamsburg-brooklyn-ny-7bd26ad8.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/chromeo/2011/terminal-5-new-york-ny-23d2c013.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/dir-en-grey/2010/nokia-theatre-times-square-new-york-ny-5bd587f8.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/dir-en-grey/2008/the-rave-eagles-club-milwaukee-wi-63d696fb.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/dir-en-grey/2008/center-stage-atlanta-ga-5bd69f68.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/dir-en-grey/2008/club-firestone-orlando-fl-33d69cf9.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/despairsray/2008/ucf-arena-orlando-fl-1bd37970.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/mucc/2008/ucf-arena-orlando-fl-bd3796e.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/dir-en-grey/2007/the-pageant-st-louis-mo-4bd6831a.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/dir-en-grey/2007/the-roxy-atlanta-ga-33d680f9.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/they-might-be-giants/2006/trustees-theater-savannah-ga-73541a31.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/the-cranberries/2002/coliseo-roberto-clemente-san-juan-puerto-rico-bd56906.html</t>
+  </si>
+  <si>
+    <t>https://www.setlist.fm/setlist/the-cranberries/2000/anfiteatro-tito-puente-san-juan-puerto-rico-bd4ad42.html</t>
   </si>
 </sst>
 </file>
@@ -543,7 +765,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -556,6 +778,14 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -576,16 +806,19 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -918,7 +1151,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8ED6F87A-CFDC-964E-A00D-12475E634363}">
-  <dimension ref="A1:K111"/>
+  <dimension ref="A1:L111"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.83203125" style="3" customWidth="1"/>
@@ -931,7 +1164,7 @@
     <col min="11" max="11" width="12.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -965,8 +1198,11 @@
       <c r="K1" s="1" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L1" s="1" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
         <v>45926</v>
       </c>
@@ -1000,8 +1236,11 @@
       <c r="K2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>45892</v>
       </c>
@@ -1035,8 +1274,11 @@
       <c r="K3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L3" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>45864</v>
       </c>
@@ -1070,8 +1312,11 @@
       <c r="K4" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L4" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>45778</v>
       </c>
@@ -1105,8 +1350,11 @@
       <c r="K5" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L5" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>45756</v>
       </c>
@@ -1137,8 +1385,11 @@
       <c r="K6" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L6" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>45755</v>
       </c>
@@ -1169,8 +1420,11 @@
       <c r="K7" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L7" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <v>45709</v>
       </c>
@@ -1205,7 +1459,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <v>45583</v>
       </c>
@@ -1239,8 +1493,11 @@
       <c r="K9" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L9" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>45553</v>
       </c>
@@ -1271,8 +1528,11 @@
       <c r="K10" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L10" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>45124</v>
       </c>
@@ -1306,8 +1566,11 @@
       <c r="K11" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L11" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>45066</v>
       </c>
@@ -1341,8 +1604,11 @@
       <c r="K12" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L12" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>45001</v>
       </c>
@@ -1376,8 +1642,11 @@
       <c r="K13" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L13" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>44960</v>
       </c>
@@ -1411,8 +1680,11 @@
       <c r="K14" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L14" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>44824</v>
       </c>
@@ -1447,7 +1719,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>44800</v>
       </c>
@@ -1482,7 +1754,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>44784</v>
       </c>
@@ -1513,8 +1785,11 @@
       <c r="K17" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L17" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>44674</v>
       </c>
@@ -1548,8 +1823,11 @@
       <c r="K18" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L18" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>44673</v>
       </c>
@@ -1583,8 +1861,11 @@
       <c r="K19" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L19" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>44470</v>
       </c>
@@ -1618,8 +1899,11 @@
       <c r="K20" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L20" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>43812</v>
       </c>
@@ -1653,8 +1937,11 @@
       <c r="K21" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L21" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>43789</v>
       </c>
@@ -1688,8 +1975,11 @@
       <c r="K22" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L22" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
         <v>43758</v>
       </c>
@@ -1720,8 +2010,11 @@
       <c r="K23" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L23" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
         <v>43757</v>
       </c>
@@ -1752,8 +2045,11 @@
       <c r="K24" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L24" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="3">
         <v>43724</v>
       </c>
@@ -1787,8 +2083,11 @@
       <c r="K25" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L25" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" s="3">
         <v>43643</v>
       </c>
@@ -1822,8 +2121,11 @@
       <c r="K26" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L26" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" s="3">
         <v>43601</v>
       </c>
@@ -1857,8 +2159,11 @@
       <c r="K27" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L27" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="3">
         <v>43597</v>
       </c>
@@ -1892,8 +2197,11 @@
       <c r="K28" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L28" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" s="3">
         <v>43576</v>
       </c>
@@ -1927,8 +2235,11 @@
       <c r="K29" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L29" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30" s="3">
         <v>43576</v>
       </c>
@@ -1962,8 +2273,11 @@
       <c r="K30" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L30" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31" s="3">
         <v>43365</v>
       </c>
@@ -1998,7 +2312,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32" s="3">
         <v>43340</v>
       </c>
@@ -2032,8 +2346,11 @@
       <c r="K32" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L32" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A33" s="3">
         <v>43194</v>
       </c>
@@ -2067,8 +2384,11 @@
       <c r="K33" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L33" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A34" s="3">
         <v>43058</v>
       </c>
@@ -2099,8 +2419,11 @@
       <c r="K34" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L34" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35" s="3">
         <v>42976</v>
       </c>
@@ -2134,8 +2457,11 @@
       <c r="K35" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L35" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A36" s="3">
         <v>42975</v>
       </c>
@@ -2169,8 +2495,11 @@
       <c r="K36" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L36" s="4" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A37" s="3">
         <v>42943</v>
       </c>
@@ -2204,10 +2533,13 @@
       <c r="K37" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L37" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A38" s="3">
-        <v>42760</v>
+        <v>42761</v>
       </c>
       <c r="B38" t="s">
         <v>164</v>
@@ -2240,7 +2572,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A39" s="3">
         <v>42761</v>
       </c>
@@ -2275,7 +2607,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A40" s="3">
         <v>42616</v>
       </c>
@@ -2309,8 +2641,11 @@
       <c r="K40" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L40" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A41" s="3">
         <v>42288</v>
       </c>
@@ -2342,7 +2677,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A42" s="3">
         <v>42224</v>
       </c>
@@ -2373,8 +2708,11 @@
       <c r="K42" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L42" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A43" s="3">
         <v>42224</v>
       </c>
@@ -2405,8 +2743,11 @@
       <c r="K43" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L43" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A44" s="3">
         <v>42224</v>
       </c>
@@ -2437,8 +2778,11 @@
       <c r="K44" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L44" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A45" s="3">
         <v>42224</v>
       </c>
@@ -2469,8 +2813,11 @@
       <c r="K45" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L45" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A46" s="3">
         <v>42167</v>
       </c>
@@ -2505,7 +2852,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A47" s="3">
         <v>42125</v>
       </c>
@@ -2539,8 +2886,11 @@
       <c r="K47" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L47" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A48" s="3">
         <v>41966</v>
       </c>
@@ -2575,7 +2925,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A49" s="3">
         <v>41958</v>
       </c>
@@ -2609,8 +2959,11 @@
       <c r="K49" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L49" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A50" s="3">
         <v>41922</v>
       </c>
@@ -2644,8 +2997,11 @@
       <c r="K50" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L50" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A51" s="3">
         <v>41905</v>
       </c>
@@ -2680,7 +3036,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A52" s="3">
         <v>41871</v>
       </c>
@@ -2714,8 +3070,11 @@
       <c r="K52" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L52" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A53" s="3">
         <v>41871</v>
       </c>
@@ -2749,8 +3108,11 @@
       <c r="K53" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L53" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A54" s="3">
         <v>41861</v>
       </c>
@@ -2781,8 +3143,11 @@
       <c r="K54" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L54" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A55" s="3">
         <v>41861</v>
       </c>
@@ -2813,8 +3178,11 @@
       <c r="K55" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L55" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A56" s="3">
         <v>41861</v>
       </c>
@@ -2845,8 +3213,11 @@
       <c r="K56" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L56" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A57" s="3">
         <v>41861</v>
       </c>
@@ -2877,8 +3248,11 @@
       <c r="K57" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L57" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A58" s="3">
         <v>41860</v>
       </c>
@@ -2909,8 +3283,11 @@
       <c r="K58" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L58" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A59" s="3">
         <v>41860</v>
       </c>
@@ -2941,8 +3318,11 @@
       <c r="K59" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L59" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A60" s="3">
         <v>41860</v>
       </c>
@@ -2973,8 +3353,11 @@
       <c r="K60" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L60" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A61" s="3">
         <v>41860</v>
       </c>
@@ -3005,8 +3388,11 @@
       <c r="K61" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L61" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A62" s="3">
         <v>41860</v>
       </c>
@@ -3037,8 +3423,11 @@
       <c r="K62" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L62" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A63" s="3">
         <v>41710</v>
       </c>
@@ -3072,8 +3461,11 @@
       <c r="K63" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L63" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A64" s="3">
         <v>41706</v>
       </c>
@@ -3108,7 +3500,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A65" s="3">
         <v>41594</v>
       </c>
@@ -3142,8 +3534,11 @@
       <c r="K65" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L65" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A66" s="3">
         <v>41222</v>
       </c>
@@ -3175,7 +3570,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A67" s="3">
         <v>41138</v>
       </c>
@@ -3206,8 +3601,11 @@
       <c r="K67" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L67" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A68" s="3">
         <v>41031</v>
       </c>
@@ -3241,8 +3639,11 @@
       <c r="K68" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L68" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A69" s="3">
         <v>40993</v>
       </c>
@@ -3276,8 +3677,11 @@
       <c r="K69" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L69" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A70" s="3">
         <v>40889</v>
       </c>
@@ -3311,8 +3715,11 @@
       <c r="K70" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L70" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="71" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A71" s="3">
         <v>40887</v>
       </c>
@@ -3343,8 +3750,11 @@
       <c r="K71" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L71" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A72" s="3">
         <v>40851</v>
       </c>
@@ -3379,7 +3789,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A73" s="3">
         <v>40847</v>
       </c>
@@ -3414,7 +3824,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A74" s="3">
         <v>40839</v>
       </c>
@@ -3448,8 +3858,11 @@
       <c r="K74" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L74" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="75" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A75" s="3">
         <v>40839</v>
       </c>
@@ -3483,8 +3896,11 @@
       <c r="K75" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L75" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="76" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A76" s="3">
         <v>40839</v>
       </c>
@@ -3518,8 +3934,11 @@
       <c r="K76" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L76" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A77" s="3">
         <v>40839</v>
       </c>
@@ -3553,8 +3972,11 @@
       <c r="K77" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L77" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="78" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A78" s="3">
         <v>40839</v>
       </c>
@@ -3588,8 +4010,11 @@
       <c r="K78" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L78" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="79" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A79" s="3">
         <v>40839</v>
       </c>
@@ -3623,8 +4048,11 @@
       <c r="K79" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L79" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="80" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A80" s="3">
         <v>40808</v>
       </c>
@@ -3658,8 +4086,11 @@
       <c r="K80" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L80" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="81" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A81" s="3">
         <v>40659</v>
       </c>
@@ -3693,8 +4124,11 @@
       <c r="K81" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L81" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="82" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A82" s="3">
         <v>40622</v>
       </c>
@@ -3728,8 +4162,11 @@
       <c r="K82" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L82" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="83" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A83" s="3">
         <v>40578</v>
       </c>
@@ -3763,8 +4200,11 @@
       <c r="K83" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L83" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="84" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A84" s="3">
         <v>40425</v>
       </c>
@@ -3795,8 +4235,11 @@
       <c r="K84" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L84" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="85" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A85" s="3">
         <v>40425</v>
       </c>
@@ -3827,8 +4270,11 @@
       <c r="K85" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L85" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="86" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A86" s="3">
         <v>40425</v>
       </c>
@@ -3859,8 +4305,11 @@
       <c r="K86" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L86" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="87" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A87" s="3">
         <v>40425</v>
       </c>
@@ -3891,8 +4340,11 @@
       <c r="K87" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L87" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="88" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A88" s="3">
         <v>40425</v>
       </c>
@@ -3923,8 +4375,11 @@
       <c r="K88" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L88" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="89" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A89" s="3">
         <v>40425</v>
       </c>
@@ -3955,8 +4410,11 @@
       <c r="K89" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L89" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="90" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A90" s="3">
         <v>40414</v>
       </c>
@@ -3990,8 +4448,11 @@
       <c r="K90" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L90" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="91" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A91" s="3">
         <v>40022</v>
       </c>
@@ -4023,7 +4484,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A92" s="3">
         <v>39955</v>
       </c>
@@ -4058,7 +4519,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A93" s="3">
         <v>39774</v>
       </c>
@@ -4089,8 +4550,11 @@
       <c r="K93" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L93" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="94" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A94" s="3">
         <v>39774</v>
       </c>
@@ -4122,7 +4586,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A95" s="3">
         <v>39760</v>
       </c>
@@ -4153,8 +4617,11 @@
       <c r="K95" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L95" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="96" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A96" s="3">
         <v>39760</v>
       </c>
@@ -4186,7 +4653,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A97" s="3">
         <v>39759</v>
       </c>
@@ -4217,8 +4684,11 @@
       <c r="K97" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L97" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="98" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A98" s="3">
         <v>39759</v>
       </c>
@@ -4250,7 +4720,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A99" s="3">
         <v>39535</v>
       </c>
@@ -4282,7 +4752,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A100" s="3">
         <v>39535</v>
       </c>
@@ -4314,7 +4784,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A101" s="3">
         <v>39535</v>
       </c>
@@ -4346,7 +4816,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A102" s="3">
         <v>39535</v>
       </c>
@@ -4377,8 +4847,11 @@
       <c r="K102" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L102" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="103" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A103" s="3">
         <v>39535</v>
       </c>
@@ -4409,8 +4882,11 @@
       <c r="K103" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L103" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="104" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A104" s="3">
         <v>39535</v>
       </c>
@@ -4442,7 +4918,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A105" s="3">
         <v>39252</v>
       </c>
@@ -4473,8 +4949,11 @@
       <c r="K105" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L105" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="106" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A106" s="3">
         <v>39252</v>
       </c>
@@ -4506,7 +4985,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A107" s="3">
         <v>39116</v>
       </c>
@@ -4537,8 +5016,11 @@
       <c r="K107" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L107" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="108" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A108" s="3">
         <v>39116</v>
       </c>
@@ -4570,7 +5052,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A109" s="3">
         <v>38841</v>
       </c>
@@ -4601,8 +5083,11 @@
       <c r="K109" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L109" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="110" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A110" s="3">
         <v>37416</v>
       </c>
@@ -4633,8 +5118,11 @@
       <c r="K110" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L110" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="111" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A111" s="3">
         <v>36623</v>
       </c>
@@ -4664,6 +5152,9 @@
       </c>
       <c r="K111" t="s">
         <v>21</v>
+      </c>
+      <c r="L111" t="s">
+        <v>238</v>
       </c>
     </row>
   </sheetData>
@@ -4672,6 +5163,9 @@
       <sortCondition descending="1" ref="A1:A111"/>
     </sortState>
   </autoFilter>
+  <hyperlinks>
+    <hyperlink ref="L36" r:id="rId1" xr:uid="{EEE27A5A-9651-204A-B510-8851DA7C7D20}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>